<commit_message>
feat(ledger): sync and record latest student ledger up to 2026-10-31
</commit_message>
<xml_diff>
--- a/成绩跟踪表.xlsx
+++ b/成绩跟踪表.xlsx
@@ -760,38 +760,98 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n"/>
-      <c r="B6" s="2" t="n"/>
-      <c r="C6" s="2" t="n"/>
-      <c r="D6" s="2" t="n"/>
-      <c r="E6" s="2" t="n"/>
-      <c r="F6" s="2" t="n"/>
+      <c r="A6" s="11" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>数学</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>期中模拟测试（校内，答卷已下发）</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>模拟考</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>67</v>
+      </c>
       <c r="G6" s="3">
         <f>IFERROR(F6/E6,"")</f>
         <v/>
       </c>
-      <c r="H6" s="2" t="n"/>
-      <c r="I6" s="2" t="n"/>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>并列第29（49人）</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>班均69.98、中位68、最高100、最低17；及格36人、≥85分12人</t>
+        </is>
+      </c>
       <c r="J6" s="4" t="n"/>
       <c r="K6" s="4" t="n"/>
       <c r="L6" s="4" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n"/>
-      <c r="B7" s="2" t="n"/>
-      <c r="C7" s="2" t="n"/>
-      <c r="D7" s="2" t="n"/>
-      <c r="E7" s="2" t="n"/>
-      <c r="F7" s="2" t="n"/>
+      <c r="A7" s="11" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>英语（蓝天）</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>课次8 课堂成绩表（宝典真题卷一/语法填空/阅读理解/词法单选/六选五）</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>机构课堂</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>135</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>110</v>
+      </c>
       <c r="G7" s="3">
         <f>IFERROR(F7/E7,"")</f>
         <v/>
       </c>
-      <c r="H7" s="2" t="n"/>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>第3（20人）</t>
+        </is>
+      </c>
       <c r="I7" s="2" t="n"/>
-      <c r="J7" s="4" t="n"/>
-      <c r="K7" s="4" t="n"/>
-      <c r="L7" s="4" t="n"/>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>真题卷一 49/60（均47）｜语法填空 16/20（均16，持平）｜阅读理解 5/5（满，均5）｜词法单选 35/40（均26，扣9分优势，全班第1）｜阅读6选5 5/10（均5，得分率仅50%，全场最低项）；总分110/135，班均96，第3名（第1名123，第2名112）</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>语法填空短板已补到班均→转为守住，每周1篇维持；六选五是唯一低于60%的项（篇章逻辑衔接），专项4篇；朗读打卡2、3未提交，本周内补齐</t>
+        </is>
+      </c>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t>U1–U2 词汇自测=已完成已签名（全班20人：9人已签名、10人未签名、1人未完成）；ClassIn 朗读打卡 94/未提交/未提交，平均94（班均91）；与第7课（155口径）不同，总分不可直接比较，仅比得分率</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n"/>
@@ -8568,7 +8628,7 @@
     </row>
     <row r="26">
       <c r="A26" s="7" t="n">
-        <v>46323</v>
+        <v>46325</v>
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
@@ -8577,12 +8637,12 @@
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>第七讲课本练习：练习3-1第5题、3-2第3题、3-4第1、3题</t>
+          <t>第七讲 A 组：练习3-1⑤、3-2③、3-4①③（原定10-28）</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>20 分钟</t>
+          <t>40 分钟</t>
         </is>
       </c>
       <c r="E26" s="6" t="inlineStr">
@@ -8597,14 +8657,18 @@
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t>本周课外；周五课前交（见 02_数学/作业记录/2026-10-30_蓝天数学第七讲课本练习_本周安排.md）</t>
-        </is>
-      </c>
-      <c r="H26" s="4" t="n"/>
+          <t>北师大第三章 整式及其加减</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t>今晚 17:30–18:10｜家长 10-30 17:26：蓝天数学明天交，今天全部完成</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="n">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
@@ -8613,12 +8677,12 @@
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>第七讲：练习3-3 全部 + 3-5第2题</t>
+          <t>第七讲 B 组：练习3-3 全部 + 3-5②（原定10-29）</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>35 分钟</t>
+          <t>40 分钟</t>
         </is>
       </c>
       <c r="E27" s="6" t="inlineStr">
@@ -8633,10 +8697,14 @@
       </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
-          <t>同上</t>
-        </is>
-      </c>
-      <c r="H27" s="4" t="n"/>
+          <t>北师大第三章 整式及其加减</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>今晚 18:20–19:00｜家长 10-30 17:26：蓝天数学明天交，今天全部完成</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="n">
@@ -8649,12 +8717,12 @@
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>第七讲：练习3-6第2题 + 练习3-7 全部 + 自查</t>
+          <t>第七讲 C 组：练习3-6② + 3-7 全部 + 自查（原定10-30）</t>
         </is>
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>45 分钟</t>
+          <t>50 分钟</t>
         </is>
       </c>
       <c r="E28" s="6" t="inlineStr">
@@ -8669,10 +8737,14 @@
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>课前完成；错题登记</t>
-        </is>
-      </c>
-      <c r="H28" s="4" t="n"/>
+          <t>北师大第三章 整式及其加减</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
+          <t>今晚 21:30–22:20｜家长 10-30 17:26：蓝天数学明天交，今天全部完成</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="n">
@@ -9131,7 +9203,7 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
+          <t>❌未完成（家长 10-28 22:34 确认）</t>
         </is>
       </c>
       <c r="F40" s="2" t="n"/>
@@ -9142,13 +9214,13 @@
       </c>
       <c r="H40" s="4" t="inlineStr">
         <is>
-          <t>老师提纲44题；答案在历史作业本上（不写提纲纸）；写完订正+家长签字；11-02上交</t>
+          <t>顺延至 10-29 晚 20:00 补做</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="11" t="n">
-        <v>46324</v>
+        <v>46326</v>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
@@ -9157,34 +9229,38 @@
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>第8课 夏商周时期的科技与文化：背诵+默写（11题）</t>
+          <t>第7课 百家争鸣（12题）+ 第8课 夏商周科技与文化（11题）：背诵+默写</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>20 分钟</t>
+          <t>40 分钟</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
-        </is>
-      </c>
-      <c r="F41" s="2" t="n"/>
+          <t>未完成</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
-          <t>第二三单元 第7-10课</t>
+          <t>写成历史作业本，不写提纲纸；老师 10-30 再次通知周一交</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr">
         <is>
-          <t>老师提纲44题；答案在历史作业本上（不写提纲纸）；写完订正+家长签字；11-02上交</t>
+          <t>10-31 09:00 段（原定 10-29，已顺延两次）</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="11" t="n">
-        <v>46325</v>
+        <v>46326</v>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
@@ -9193,28 +9269,32 @@
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>第9课 秦统一中国：背诵+默写（14题）</t>
+          <t>第9课 秦统一中国（14题）：背诵+默写</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>20 分钟</t>
+          <t>25 分钟</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
-        </is>
-      </c>
-      <c r="F42" s="2" t="n"/>
+          <t>未完成</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
-          <t>第二三单元 第7-10课</t>
+          <t>三公职权、郡县制vs分封制、公元前221年</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr">
         <is>
-          <t>老师提纲44题；答案在历史作业本上（不写提纲纸）；写完订正+家长签字；11-02上交</t>
+          <t>10-31 14:30 段</t>
         </is>
       </c>
     </row>
@@ -9229,28 +9309,32 @@
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>第10课 秦末农民大起义：背诵+默写（7题）</t>
+          <t>第10课 秦末农民大起义（7题）：背诵+默写</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>20 分钟</t>
+          <t>15 分钟</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
-        </is>
-      </c>
-      <c r="F43" s="2" t="n"/>
+          <t>未完成</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G43" s="4" t="inlineStr">
         <is>
-          <t>第二三单元 第7-10课</t>
+          <t>陈胜起义直接原因(遇雨失期)与根本原因(秦的暴政)</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr">
         <is>
-          <t>老师提纲44题；答案在历史作业本上（不写提纲纸）；写完订正+家长签字；11-02上交</t>
+          <t>10-31 14:30 段</t>
         </is>
       </c>
     </row>
@@ -9265,12 +9349,12 @@
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>期中复习：第7-10课 错题重默（本周不再排新课）</t>
+          <t>四课 44 题抽背 + 家长签字（签「已背已默」）</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>20 分钟</t>
+          <t>45 分钟</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
@@ -9278,15 +9362,19 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="F44" s="2" t="n"/>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G44" s="4" t="inlineStr">
         <is>
-          <t>第二三单元 第7-10课</t>
+          <t>答不出画圈，只重背圈出的；11-02 上交</t>
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr">
         <is>
-          <t>老师提纲44题；答案在历史作业本上（不写提纲纸）；写完订正+家长签字；11-02上交</t>
+          <t>11-01 10:00 段</t>
         </is>
       </c>
     </row>
@@ -9371,24 +9459,84 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="n"/>
-      <c r="B47" s="2" t="n"/>
-      <c r="C47" s="4" t="n"/>
-      <c r="D47" s="2" t="n"/>
-      <c r="E47" s="2" t="n"/>
-      <c r="F47" s="2" t="n"/>
-      <c r="G47" s="4" t="n"/>
-      <c r="H47" s="4" t="n"/>
+      <c r="A47" s="11" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>数学</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>第四章 基本平面图形 第2课时 P77–P78（共18题）</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>30 分钟</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>已完成（已批改）</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>18题错4题（P77第4、9(1)；P78第13、15(2)②）</t>
+        </is>
+      </c>
+      <c r="G47" s="4" t="inlineStr">
+        <is>
+          <t>叠合法三种实现；线段中点比例关系</t>
+        </is>
+      </c>
+      <c r="H47" s="4" t="inlineStr">
+        <is>
+          <t>批改稿 02_数学/作业记录/2026-10-28_第四章第2课时_P77_批改.md（两页均已批）</t>
+        </is>
+      </c>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="n"/>
-      <c r="B48" s="2" t="n"/>
-      <c r="C48" s="4" t="n"/>
-      <c r="D48" s="2" t="n"/>
-      <c r="E48" s="2" t="n"/>
-      <c r="F48" s="2" t="n"/>
-      <c r="G48" s="4" t="n"/>
-      <c r="H48" s="4" t="n"/>
+      <c r="A48" s="11" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>生物</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>第一单元（第二章）知识加油站 全卷（选择1–30、非选择31–34）</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>15 分钟</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>已完成（已批改）</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>选择30题对16错5空8；31题空3；32题对8错3；33题空6；34题对4错1；空白共17处</t>
+        </is>
+      </c>
+      <c r="G48" s="4" t="inlineStr">
+        <is>
+          <t>短板：植物器官辨识、结构层次顺序、四种组织功能；空白题成片出现需确认是否做完</t>
+        </is>
+      </c>
+      <c r="H48" s="4" t="inlineStr">
+        <is>
+          <t>批改稿 04_生物/作业记录/2026-10-28_第二章知识加油站_选择题_批改.md；空白11处待补</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n"/>
@@ -9401,214 +9549,820 @@
       <c r="H49" s="4" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="n"/>
-      <c r="B50" s="2" t="n"/>
-      <c r="C50" s="4" t="n"/>
-      <c r="D50" s="2" t="n"/>
-      <c r="E50" s="2" t="n"/>
-      <c r="F50" s="2" t="n"/>
-      <c r="G50" s="4" t="n"/>
-      <c r="H50" s="4" t="n"/>
+      <c r="A50" s="11" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>英语</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>蓝天宝典 U1 词性转换默写（P11，12组22空）</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>15 分钟</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>已完成（家长 10-28 22:19，拍照）</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>22 空对 20，明确错 1 处（improve→improvement），约 95%</t>
+        </is>
+      </c>
+      <c r="G50" s="4" t="inlineStr">
+        <is>
+          <t>动词+(-ment)变名词；person 单数</t>
+        </is>
+      </c>
+      <c r="H50" s="4" t="inlineStr">
+        <is>
+          <t>批改稿 03_英语/语法/2026-10-28_蓝天宝典_U1词性转换_12组22空_默写批改.md</t>
+        </is>
+      </c>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="n"/>
-      <c r="B51" s="2" t="n"/>
-      <c r="C51" s="4" t="n"/>
-      <c r="D51" s="2" t="n"/>
-      <c r="E51" s="2" t="n"/>
-      <c r="F51" s="2" t="n"/>
-      <c r="G51" s="4" t="n"/>
-      <c r="H51" s="4" t="n"/>
+      <c r="A51" s="11" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>英语</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>前三单元作文描红（衡水体字帖，家长已打印）</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>明天带回学校（老师统一安排）</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>材料已打印（家中），明天带回</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G51" s="4" t="inlineStr">
+        <is>
+          <t>衡水体书写；U1-U3 作文句型</t>
+        </is>
+      </c>
+      <c r="H51" s="4" t="inlineStr">
+        <is>
+          <t>老师 10-29 15:48 明确：家长打印后转交孩子，**明天(10-30)上课带回**；今晚不描</t>
+        </is>
+      </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="n"/>
-      <c r="B52" s="2" t="n"/>
-      <c r="C52" s="4" t="n"/>
-      <c r="D52" s="2" t="n"/>
-      <c r="E52" s="2" t="n"/>
-      <c r="F52" s="2" t="n"/>
-      <c r="G52" s="4" t="n"/>
-      <c r="H52" s="4" t="n"/>
+      <c r="A52" s="11" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>英语</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>蓝天宝典 U1–U2 四面全部必交：①U1词性转换 ②U1短语+英英释义 ③U2词性转换 ④U2短语+英英释义</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>约 120 分钟（分 3 段）</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>已完成（家长 10-30 20:53：蓝天英语全部写完）</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>待签字</t>
+        </is>
+      </c>
+      <c r="G52" s="4" t="inlineStr">
+        <is>
+          <t>词性转换 / 后缀 -ment -ness -ence 类</t>
+        </is>
+      </c>
+      <c r="H52" s="4" t="inlineStr">
+        <is>
+          <t>四面交齐：①②③④均已完成；明早抽查+签字后上交</t>
+        </is>
+      </c>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="n"/>
-      <c r="B53" s="2" t="n"/>
-      <c r="C53" s="4" t="n"/>
-      <c r="D53" s="2" t="n"/>
-      <c r="E53" s="2" t="n"/>
-      <c r="F53" s="2" t="n"/>
-      <c r="G53" s="4" t="n"/>
-      <c r="H53" s="4" t="n"/>
+      <c r="A53" s="11" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>英语</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>宝典签名前抽查 5 词（合书限时 10 秒/词）</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>2 分钟</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>待做（明早 08:20 抽查签字）</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G53" s="4" t="inlineStr">
+        <is>
+          <t>honesty / improvement / relaxed / lucky / careless</t>
+        </is>
+      </c>
+      <c r="H53" s="4" t="inlineStr">
+        <is>
+          <t>抽查卡：00_台账规范/宝典默写抽查卡_A4.docx</t>
+        </is>
+      </c>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="n"/>
-      <c r="B54" s="2" t="n"/>
-      <c r="C54" s="4" t="n"/>
-      <c r="D54" s="2" t="n"/>
-      <c r="E54" s="2" t="n"/>
-      <c r="F54" s="2" t="n"/>
-      <c r="G54" s="4" t="n"/>
-      <c r="H54" s="4" t="n"/>
+      <c r="A54" s="11" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>英语</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>宝典 ③U2 词性转换（P13–P14）默写+订正</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>40 分钟</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>已完成（家长 10-30 20:53：蓝天英语全部写完）</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G54" s="4" t="inlineStr">
+        <is>
+          <t>-ence/-ment/-ly 类后缀</t>
+        </is>
+      </c>
+      <c r="H54" s="4" t="inlineStr">
+        <is>
+          <t>今晚 17:30–18:10｜先背 10′→合书默→红笔圈错→错词再默</t>
+        </is>
+      </c>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="n"/>
-      <c r="B55" s="2" t="n"/>
-      <c r="C55" s="4" t="n"/>
-      <c r="D55" s="2" t="n"/>
-      <c r="E55" s="2" t="n"/>
-      <c r="F55" s="2" t="n"/>
-      <c r="G55" s="4" t="n"/>
-      <c r="H55" s="4" t="n"/>
+      <c r="A55" s="11" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>英语</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t>宝典 ②U1 短语+英英释义（英→中 + 中→英 双向）</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>40 分钟</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>已完成（家长 10-30 20:53：蓝天英语全部写完）</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G55" s="4" t="inlineStr">
+        <is>
+          <t>短语固定搭配 / 英文释义</t>
+        </is>
+      </c>
+      <c r="H55" s="4" t="inlineStr">
+        <is>
+          <t>今晚 18:10–18:50｜释义背英文例句，不背中文</t>
+        </is>
+      </c>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="n"/>
-      <c r="B56" s="2" t="n"/>
-      <c r="C56" s="4" t="n"/>
-      <c r="D56" s="2" t="n"/>
-      <c r="E56" s="2" t="n"/>
-      <c r="F56" s="2" t="n"/>
-      <c r="G56" s="4" t="n"/>
-      <c r="H56" s="4" t="n"/>
+      <c r="A56" s="11" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>英语</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>宝典 ④U2 短语+英英释义</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>45 分钟</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>已完成（家长 10-30 20:53：蓝天英语全部写完）</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G56" s="4" t="inlineStr">
+        <is>
+          <t>短语固定搭配 / 英文释义</t>
+        </is>
+      </c>
+      <c r="H56" s="4" t="inlineStr">
+        <is>
+          <t>数学课后 21:00–21:45｜英→中先过，中→英只做标粗与错过的</t>
+        </is>
+      </c>
     </row>
     <row r="57">
-      <c r="A57" s="2" t="n"/>
-      <c r="B57" s="2" t="n"/>
-      <c r="C57" s="4" t="n"/>
-      <c r="D57" s="2" t="n"/>
-      <c r="E57" s="2" t="n"/>
-      <c r="F57" s="2" t="n"/>
-      <c r="G57" s="4" t="n"/>
-      <c r="H57" s="4" t="n"/>
+      <c r="A57" s="11" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>英语</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>宝典四面 抽查 5 词 + 家长签字</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>5 分钟</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>待做（明早 08:20）</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G57" s="4" t="inlineStr">
+        <is>
+          <t>抽 honesty/improvement/confident/patience/impatiently</t>
+        </is>
+      </c>
+      <c r="H57" s="4" t="inlineStr">
+        <is>
+          <t>21:45–21:50｜签字写「已默写」+ 日期</t>
+        </is>
+      </c>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="n"/>
-      <c r="B58" s="2" t="n"/>
-      <c r="C58" s="4" t="n"/>
-      <c r="D58" s="2" t="n"/>
-      <c r="E58" s="2" t="n"/>
-      <c r="F58" s="2" t="n"/>
-      <c r="G58" s="4" t="n"/>
-      <c r="H58" s="4" t="n"/>
+      <c r="A58" s="11" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>英语</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>宝典①：U3–U4 词汇短语 背记+默写（P15–18）+ 红笔订正 + 家长签名</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>40 分钟</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>待做</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G58" s="4" t="inlineStr">
+        <is>
+          <t>U3–U4 词汇 / 词性 / 短语搭配</t>
+        </is>
+      </c>
+      <c r="H58" s="4" t="inlineStr">
+        <is>
+          <t>蓝天英语第8课作业1｜下节课检查（❓11-07 周六）｜先背10′→合书默→红笔订正→错词再默</t>
+        </is>
+      </c>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="n"/>
-      <c r="B59" s="2" t="n"/>
-      <c r="C59" s="4" t="n"/>
-      <c r="D59" s="2" t="n"/>
-      <c r="E59" s="2" t="n"/>
-      <c r="F59" s="2" t="n"/>
-      <c r="G59" s="4" t="n"/>
-      <c r="H59" s="4" t="n"/>
+      <c r="A59" s="11" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>英语</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>宝典②：阅读理解 3–4 篇（P39–41）</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>25 分钟</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>待做</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G59" s="4" t="inlineStr">
+        <is>
+          <t>细节 / 主旨 / 推断 / 指代</t>
+        </is>
+      </c>
+      <c r="H59" s="4" t="inlineStr">
+        <is>
+          <t>蓝天英语第8课作业2｜建议 11-01 与六选五连做，限时45′</t>
+        </is>
+      </c>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="n"/>
-      <c r="B60" s="2" t="n"/>
-      <c r="C60" s="4" t="n"/>
-      <c r="D60" s="2" t="n"/>
-      <c r="E60" s="2" t="n"/>
-      <c r="F60" s="2" t="n"/>
-      <c r="G60" s="4" t="n"/>
-      <c r="H60" s="4" t="n"/>
+      <c r="A60" s="11" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>英语</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="inlineStr">
+        <is>
+          <t>宝典③：六选五 3–4 篇（P43–44）</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>20 分钟</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>待做</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G60" s="4" t="inlineStr">
+        <is>
+          <t>篇章衔接 / 逻辑关系</t>
+        </is>
+      </c>
+      <c r="H60" s="4" t="inlineStr">
+        <is>
+          <t>蓝天英语第8课作业3｜与阅读理解连做，按考试节奏</t>
+        </is>
+      </c>
     </row>
     <row r="61">
-      <c r="A61" s="2" t="n"/>
-      <c r="B61" s="2" t="n"/>
-      <c r="C61" s="4" t="n"/>
-      <c r="D61" s="2" t="n"/>
-      <c r="E61" s="2" t="n"/>
-      <c r="F61" s="2" t="n"/>
-      <c r="G61" s="4" t="n"/>
-      <c r="H61" s="4" t="n"/>
+      <c r="A61" s="11" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>英语</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t>宝典④：AEG U3 范文——进阶版 背记（P55）</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>25 分钟</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>待做</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G61" s="4" t="inlineStr">
+        <is>
+          <t>句式储备 / 主谓一致 / 句子缺谓语</t>
+        </is>
+      </c>
+      <c r="H61" s="4" t="inlineStr">
+        <is>
+          <t>蓝天英语第8课作业4｜关键词框架法，拆3段；对应10-28作文9处错误</t>
+        </is>
+      </c>
     </row>
     <row r="62">
-      <c r="A62" s="2" t="n"/>
-      <c r="B62" s="2" t="n"/>
-      <c r="C62" s="4" t="n"/>
-      <c r="D62" s="2" t="n"/>
-      <c r="E62" s="2" t="n"/>
-      <c r="F62" s="2" t="n"/>
-      <c r="G62" s="4" t="n"/>
-      <c r="H62" s="4" t="n"/>
+      <c r="A62" s="11" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>英语</t>
+        </is>
+      </c>
+      <c r="C62" s="4" t="inlineStr">
+        <is>
+          <t>朗读打卡 3 次</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>30 分钟（3×10）</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>待做</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G62" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H62" s="4" t="inlineStr">
+        <is>
+          <t>蓝天英语第8课作业5｜建议 11-01/03/05 各一次，别攒到最后</t>
+        </is>
+      </c>
     </row>
     <row r="63">
-      <c r="A63" s="2" t="n"/>
-      <c r="B63" s="2" t="n"/>
-      <c r="C63" s="4" t="n"/>
-      <c r="D63" s="2" t="n"/>
-      <c r="E63" s="2" t="n"/>
-      <c r="F63" s="2" t="n"/>
-      <c r="G63" s="4" t="n"/>
-      <c r="H63" s="4" t="n"/>
+      <c r="A63" s="11" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>数学</t>
+        </is>
+      </c>
+      <c r="C63" s="4" t="inlineStr">
+        <is>
+          <t>校内周末作业：数学试卷 2 份</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>80 分钟</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>待做</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G63" s="4" t="inlineStr">
+        <is>
+          <t>❓待定（拿到卷子后登记）</t>
+        </is>
+      </c>
+      <c r="H63" s="4" t="inlineStr">
+        <is>
+          <t>11-06 数学期中｜家长 14:28 更正：**2 份试卷**（原记 4 页已更正）；分两天各 40′ 限时；❓卷名待确认；10-31 第1份 / 11-01 第2份</t>
+        </is>
+      </c>
     </row>
     <row r="64">
-      <c r="A64" s="2" t="n"/>
-      <c r="B64" s="2" t="n"/>
-      <c r="C64" s="4" t="n"/>
-      <c r="D64" s="2" t="n"/>
-      <c r="E64" s="2" t="n"/>
-      <c r="F64" s="2" t="n"/>
-      <c r="G64" s="4" t="n"/>
-      <c r="H64" s="4" t="n"/>
+      <c r="A64" s="11" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>生物</t>
+        </is>
+      </c>
+      <c r="C64" s="4" t="inlineStr">
+        <is>
+          <t>校内周末作业①：考试试卷重新做</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>40 分钟</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>待做</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G64" s="4" t="inlineStr">
+        <is>
+          <t>❓待定（对照第一次错处）</t>
+        </is>
+      </c>
+      <c r="H64" s="4" t="inlineStr">
+        <is>
+          <t>11-06 生地合卷｜目标卷=10-27 期中模拟考（第1–3章/满分50/40分钟），用 2026-10-30 空白卷 PDF 重做；家长确认未及格；❓具体分数待补</t>
+        </is>
+      </c>
     </row>
     <row r="65">
-      <c r="A65" s="2" t="n"/>
-      <c r="B65" s="2" t="n"/>
-      <c r="C65" s="4" t="n"/>
-      <c r="D65" s="2" t="n"/>
-      <c r="E65" s="2" t="n"/>
-      <c r="F65" s="2" t="n"/>
-      <c r="G65" s="4" t="n"/>
-      <c r="H65" s="4" t="n"/>
+      <c r="A65" s="11" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>生物</t>
+        </is>
+      </c>
+      <c r="C65" s="4" t="inlineStr">
+        <is>
+          <t>校内周末作业②：复习资料全部仔细过一遍</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>30 分钟</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>待做</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G65" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H65" s="4" t="inlineStr">
+        <is>
+          <t>11-06 生地合卷｜10-17 小测 10/20（班均14.08）为已知薄弱</t>
+        </is>
+      </c>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="n"/>
-      <c r="B66" s="2" t="n"/>
-      <c r="C66" s="4" t="n"/>
-      <c r="D66" s="2" t="n"/>
-      <c r="E66" s="2" t="n"/>
-      <c r="F66" s="2" t="n"/>
-      <c r="G66" s="4" t="n"/>
-      <c r="H66" s="4" t="n"/>
+      <c r="A66" s="11" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>历史</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t>校内周末作业：4 课背→默写→订正→家长签字</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>60 分钟</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>待做</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G66" s="4" t="inlineStr">
+        <is>
+          <t>❓哪 4 课待确认（疑第1–4课）</t>
+        </is>
+      </c>
+      <c r="H66" s="4" t="inlineStr">
+        <is>
+          <t>11-05 历史期中｜一课15′（背5′+默+改+签），默写纸留存｜家长 14:40 确认：默写本 11-02 周一照交，与「1 份试卷」两项都要交</t>
+        </is>
+      </c>
     </row>
     <row r="67">
-      <c r="A67" s="2" t="n"/>
-      <c r="B67" s="2" t="n"/>
-      <c r="C67" s="4" t="n"/>
-      <c r="D67" s="2" t="n"/>
-      <c r="E67" s="2" t="n"/>
-      <c r="F67" s="2" t="n"/>
-      <c r="G67" s="4" t="n"/>
-      <c r="H67" s="4" t="n"/>
+      <c r="A67" s="11" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>地理</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="inlineStr">
+        <is>
+          <t>校内周末作业：老师发的复习材料过一遍</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>20 分钟</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>待做</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G67" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H67" s="4" t="inlineStr">
+        <is>
+          <t>11-06 生地合卷｜⚠️材料未收到，需家长转发</t>
+        </is>
+      </c>
     </row>
     <row r="68">
-      <c r="A68" s="2" t="n"/>
-      <c r="B68" s="2" t="n"/>
-      <c r="C68" s="4" t="n"/>
-      <c r="D68" s="2" t="n"/>
-      <c r="E68" s="2" t="n"/>
+      <c r="A68" s="11" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>语文</t>
+        </is>
+      </c>
+      <c r="C68" s="4" t="inlineStr">
+        <is>
+          <t>校内周末作业：试卷 1 份</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>45 分钟</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>待做</t>
+        </is>
+      </c>
       <c r="F68" s="2" t="n"/>
       <c r="G68" s="4" t="n"/>
-      <c r="H68" s="4" t="n"/>
+      <c r="H68" s="4" t="inlineStr">
+        <is>
+          <t>11-05 语文期中｜❓哪份卷、含不含作文；排 10-31 16:20（若含作文需加时）</t>
+        </is>
+      </c>
     </row>
     <row r="69">
-      <c r="A69" s="2" t="n"/>
-      <c r="B69" s="2" t="n"/>
-      <c r="C69" s="4" t="n"/>
-      <c r="D69" s="2" t="n"/>
-      <c r="E69" s="2" t="n"/>
+      <c r="A69" s="11" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>英语</t>
+        </is>
+      </c>
+      <c r="C69" s="4" t="inlineStr">
+        <is>
+          <t>校内周末作业：听说</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>25 分钟</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>待做</t>
+        </is>
+      </c>
       <c r="F69" s="2" t="n"/>
       <c r="G69" s="4" t="n"/>
-      <c r="H69" s="4" t="n"/>
+      <c r="H69" s="4" t="inlineStr">
+        <is>
+          <t>11-06 英语｜平台 **E 听说 App**（与之前相同：老师开放后登录、一次录音）；❓几套/截止（以往 21:30 硬截止）；排 11-01 20:40</t>
+        </is>
+      </c>
     </row>
     <row r="70">
-      <c r="A70" s="2" t="n"/>
-      <c r="B70" s="2" t="n"/>
-      <c r="C70" s="4" t="n"/>
-      <c r="D70" s="2" t="n"/>
-      <c r="E70" s="2" t="n"/>
+      <c r="A70" s="11" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>历史</t>
+        </is>
+      </c>
+      <c r="C70" s="4" t="inlineStr">
+        <is>
+          <t>校内周末作业：试卷 1 份</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>35 分钟</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>待做</t>
+        </is>
+      </c>
       <c r="F70" s="2" t="n"/>
       <c r="G70" s="4" t="n"/>
-      <c r="H70" s="4" t="n"/>
+      <c r="H70" s="4" t="inlineStr">
+        <is>
+          <t>11-05 历史期中｜❓卷名待确认；与「4 课背默」并行，默写本 11-02 交；排 11-01 10:20</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n"/>
@@ -10011,7 +10765,7 @@
       <c r="H110" s="4" t="n"/>
     </row>
     <row r="111">
-      <c r="A111" s="2" t="n"/>
+      <c r="A111" s="11" t="n"/>
       <c r="B111" s="2" t="n"/>
       <c r="C111" s="4" t="n"/>
       <c r="D111" s="2" t="n"/>
@@ -10021,7 +10775,7 @@
       <c r="H111" s="4" t="n"/>
     </row>
     <row r="112">
-      <c r="A112" s="2" t="n"/>
+      <c r="A112" s="11" t="n"/>
       <c r="B112" s="2" t="n"/>
       <c r="C112" s="4" t="n"/>
       <c r="D112" s="2" t="n"/>
@@ -18165,498 +18919,1822 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="n"/>
-      <c r="B25" s="2" t="n"/>
-      <c r="C25" s="2" t="n"/>
-      <c r="D25" s="2" t="n"/>
-      <c r="E25" s="4" t="n"/>
-      <c r="F25" s="4" t="n"/>
-      <c r="G25" s="4" t="n"/>
-      <c r="H25" s="2" t="n"/>
-      <c r="I25" s="2" t="n"/>
+      <c r="A25" s="11" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>语文</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>10-27 语文作业：词语注音抄写（6词×3遍）</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>凋零（3遍全错）</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>前后鼻音 in/ing：零 líng</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>前后鼻音不分，用 lín 代替 líng</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>正确 diāo líng；零＝后鼻音，-ng 要念满</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>❌未掌握</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
       <c r="J25" s="2" t="n"/>
       <c r="K25" s="4" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="n"/>
-      <c r="B26" s="2" t="n"/>
-      <c r="C26" s="2" t="n"/>
-      <c r="D26" s="2" t="n"/>
-      <c r="E26" s="4" t="n"/>
-      <c r="F26" s="4" t="n"/>
-      <c r="G26" s="4" t="n"/>
-      <c r="H26" s="2" t="n"/>
-      <c r="I26" s="2" t="n"/>
+      <c r="A26" s="11" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>语文</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>10-27 语文作业：词语注音抄写</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>枯萎（3遍全错）</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>形近字：萎（艹）vs 燥（火）</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>按读音记词未看字形，抄3遍仍写错</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>正确 kū wěi；燥＝干燥（火），萎＝枯萎（艹）</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>❌未掌握</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
       <c r="J26" s="2" t="n"/>
       <c r="K26" s="4" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="n"/>
-      <c r="B27" s="2" t="n"/>
-      <c r="C27" s="2" t="n"/>
-      <c r="D27" s="2" t="n"/>
-      <c r="E27" s="4" t="n"/>
-      <c r="F27" s="4" t="n"/>
-      <c r="G27" s="4" t="n"/>
-      <c r="H27" s="2" t="n"/>
-      <c r="I27" s="2" t="n"/>
+      <c r="A27" s="11" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>语文</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>10-27 语文作业：词语注音抄写</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>喧嚷（3遍全错）</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>嚷 rǎng 三声，与闹 nào 混淆</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>音近词混用</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>正确 xuān rǎng；嚷＝口＋襄，三声</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>❌未掌握</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
       <c r="J27" s="2" t="n"/>
       <c r="K27" s="4" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="n"/>
-      <c r="B28" s="2" t="n"/>
-      <c r="C28" s="2" t="n"/>
-      <c r="D28" s="2" t="n"/>
-      <c r="E28" s="4" t="n"/>
-      <c r="F28" s="4" t="n"/>
-      <c r="G28" s="4" t="n"/>
-      <c r="H28" s="2" t="n"/>
-      <c r="I28" s="2" t="n"/>
+      <c r="A28" s="11" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>语文</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>10-27 语文作业：词语注音抄写</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>邀请（3遍错2）</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>请 qǐng 三声</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>声调靠蒙，同一词三遍写三个调</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>正确 yāo qǐng；请＝三声</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>⚠️部分掌握</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
       <c r="J28" s="2" t="n"/>
       <c r="K28" s="4" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="n"/>
-      <c r="B29" s="2" t="n"/>
-      <c r="C29" s="2" t="n"/>
-      <c r="D29" s="2" t="n"/>
-      <c r="E29" s="4" t="n"/>
-      <c r="F29" s="4" t="n"/>
-      <c r="G29" s="4" t="n"/>
-      <c r="H29" s="2" t="n"/>
-      <c r="I29" s="2" t="n"/>
+      <c r="A29" s="11" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>语文</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>10-27 语文作业：抄写《西游记》第二回片段</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>参禅打坐、戒语持斋</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>听音写字：参禅→各种；戒语→或语</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>抄写不看原文，凭听感写</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>正确：参禅打坐、戒语持斋（祖师答悟空语）</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>❌未掌握</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
       <c r="J29" s="2" t="n"/>
       <c r="K29" s="4" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="n"/>
-      <c r="B30" s="2" t="n"/>
-      <c r="C30" s="2" t="n"/>
-      <c r="D30" s="2" t="n"/>
-      <c r="E30" s="4" t="n"/>
-      <c r="F30" s="4" t="n"/>
-      <c r="G30" s="4" t="n"/>
-      <c r="H30" s="2" t="n"/>
-      <c r="I30" s="2" t="n"/>
+      <c r="A30" s="11" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>道法</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>10-26 道法「最美家庭」小文观点题（12分）</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>全题（约5/12）</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>材料题三步法：判断→分析→分主体建议</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>不答错在哪、完全不给建议、通篇不用材料</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>①判断片面＋理由 ②结合材料分两面 ③建议分小文/爸爸/妈妈/全家</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>❌未掌握</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-04</t>
+        </is>
+      </c>
       <c r="J30" s="2" t="n"/>
       <c r="K30" s="4" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="n"/>
-      <c r="B31" s="2" t="n"/>
-      <c r="C31" s="2" t="n"/>
-      <c r="D31" s="2" t="n"/>
-      <c r="E31" s="4" t="n"/>
-      <c r="F31" s="4" t="n"/>
-      <c r="G31" s="4" t="n"/>
-      <c r="H31" s="2" t="n"/>
-      <c r="I31" s="2" t="n"/>
+      <c r="A31" s="11" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>数学</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>10-28 校内数学作业：第四章第2课时 P77 基础题</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>第4题（选择）</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>比较线段长短的方法；叠合法有三种实现（测量/圆规/折叠）</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>漏判折叠法：只承认测量和圆规两种，误选C（2个）</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>正确 D（3个）：①刻度尺测量 ②圆规叠放 ③沿∠A角平分线折叠使AB与AC重合，看B落点</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>❌未掌握</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
       <c r="J31" s="2" t="n"/>
       <c r="K31" s="4" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="n"/>
-      <c r="B32" s="2" t="n"/>
-      <c r="C32" s="2" t="n"/>
-      <c r="D32" s="2" t="n"/>
-      <c r="E32" s="4" t="n"/>
-      <c r="F32" s="4" t="n"/>
-      <c r="G32" s="4" t="n"/>
-      <c r="H32" s="2" t="n"/>
-      <c r="I32" s="2" t="n"/>
+      <c r="A32" s="11" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>数学</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>10-28 校内数学作业：第四章第2课时 P77 基础题</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>第9题(1) 第二空</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>线段中点与线段和差的比例关系（设未知数）</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>未设元，凭直觉填；未检查大小关系（减完只会更短，不可能等于更长的AB）</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>正确 BQ。设QC=x，BC=2BQ且QB+BC=x → QB=x/3，AQ−BC=x−2x/3=x/3=BQ</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>❌未掌握</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
       <c r="J32" s="2" t="n"/>
       <c r="K32" s="4" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="n"/>
-      <c r="B33" s="2" t="n"/>
-      <c r="C33" s="2" t="n"/>
-      <c r="D33" s="2" t="n"/>
-      <c r="E33" s="4" t="n"/>
-      <c r="F33" s="4" t="n"/>
-      <c r="G33" s="4" t="n"/>
-      <c r="H33" s="2" t="n"/>
-      <c r="I33" s="2" t="n"/>
+      <c r="A33" s="11" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>数学</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>10-28 校内数学作业：第四章第2课时 P78</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>第13题</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>数轴上两点距离+线段中点（分类讨论）</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>漏负方向解；且求的是AC中点，他只算到C（填了C的坐标1）</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>正确 0 或 −2。B=−1+4=3时C=1,D=0；B=−1−4=−5时C=−3,D=−2</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>❌未掌握</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
       <c r="J33" s="2" t="n"/>
       <c r="K33" s="4" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="n"/>
-      <c r="B34" s="2" t="n"/>
-      <c r="C34" s="2" t="n"/>
-      <c r="D34" s="2" t="n"/>
-      <c r="E34" s="4" t="n"/>
-      <c r="F34" s="4" t="n"/>
-      <c r="G34" s="4" t="n"/>
-      <c r="H34" s="2" t="n"/>
-      <c r="I34" s="2" t="n"/>
+      <c r="A34" s="11" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>数学</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>10-28 校内数学作业：第四章第2课时 P78</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>第15题(2)②</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>直线上四点的位置关系与线段和</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>未画图定位，BC被重复计算（3+2+2）</t>
+        </is>
+      </c>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>正确 5cm。D—A—B—C，AD=4,AB=2,BC=2；BD=6,BP=3，CP=BP+BC=3+2=5</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>❌未掌握</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
       <c r="J34" s="2" t="n"/>
       <c r="K34" s="4" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="n"/>
-      <c r="B35" s="2" t="n"/>
-      <c r="C35" s="2" t="n"/>
-      <c r="D35" s="2" t="n"/>
-      <c r="E35" s="4" t="n"/>
-      <c r="F35" s="4" t="n"/>
-      <c r="G35" s="4" t="n"/>
-      <c r="H35" s="2" t="n"/>
-      <c r="I35" s="2" t="n"/>
+      <c r="A35" s="11" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>生物</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>10-28 生物作业：第二章知识加油站 选择题</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>第5题</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>细胞分化 vs 细胞癌变</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>把干细胞形成组织的分化过程误判为癌变</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>正确 C 细胞分化：形态结构功能改变形成组织；癌变是不受控增殖形成肿瘤</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>❌未掌握</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
       <c r="J35" s="2" t="n"/>
       <c r="K35" s="4" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="n"/>
-      <c r="B36" s="2" t="n"/>
-      <c r="C36" s="2" t="n"/>
-      <c r="D36" s="2" t="n"/>
-      <c r="E36" s="4" t="n"/>
-      <c r="F36" s="4" t="n"/>
-      <c r="G36" s="4" t="n"/>
-      <c r="H36" s="2" t="n"/>
-      <c r="I36" s="2" t="n"/>
+      <c r="A36" s="11" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>生物</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>10-28 生物作业：第二章知识加油站 选择题</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>第10题</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>植物器官的辨识（根/茎/叶/花/果）</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>大白菜误判为花；萝卜莴笋未理清</t>
+        </is>
+      </c>
+      <c r="G36" s="4" t="inlineStr">
+        <is>
+          <t>正确 B 根、茎、叶：萝卜=肉质直根，莴笋=肉质茎，大白菜=叶球</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>❌未掌握</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
       <c r="J36" s="2" t="n"/>
       <c r="K36" s="4" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="n"/>
-      <c r="B37" s="2" t="n"/>
-      <c r="C37" s="2" t="n"/>
-      <c r="D37" s="2" t="n"/>
-      <c r="E37" s="4" t="n"/>
-      <c r="F37" s="4" t="n"/>
-      <c r="G37" s="4" t="n"/>
-      <c r="H37" s="2" t="n"/>
-      <c r="I37" s="2" t="n"/>
+      <c r="A37" s="11" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>生物</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>10-28 生物作业：第二章知识加油站 选择题</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>第6题</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>动物结构层次（细胞→组织→器官→系统→个体）</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>空白未作答；层次名称与顺序不清</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>正确 C：甲=组织，乙=器官，丙=系统；分化发生在细胞→组织这一步</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>❌未掌握</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
       <c r="J37" s="2" t="n"/>
       <c r="K37" s="4" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="n"/>
-      <c r="B38" s="2" t="n"/>
-      <c r="C38" s="2" t="n"/>
-      <c r="D38" s="2" t="n"/>
-      <c r="E38" s="4" t="n"/>
-      <c r="F38" s="4" t="n"/>
-      <c r="G38" s="4" t="n"/>
-      <c r="H38" s="2" t="n"/>
-      <c r="I38" s="2" t="n"/>
+      <c r="A38" s="11" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>生物</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>10-28 生物作业：第二章知识加油站 选择题</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>第8、9题</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>四种组织的辨认（血液=结缔组织；皮肤含上皮+结缔+神经）</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>空白未作答；不知血液属结缔组织</t>
+        </is>
+      </c>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>第8题 C 上皮+结缔+神经（注意「保护组织」是植物组织名）；第9题 C 血液=结缔组织</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>❌未掌握</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
       <c r="J38" s="2" t="n"/>
       <c r="K38" s="4" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="n"/>
-      <c r="B39" s="2" t="n"/>
-      <c r="C39" s="2" t="n"/>
-      <c r="D39" s="2" t="n"/>
-      <c r="E39" s="4" t="n"/>
-      <c r="F39" s="4" t="n"/>
-      <c r="G39" s="4" t="n"/>
-      <c r="H39" s="2" t="n"/>
-      <c r="I39" s="2" t="n"/>
+      <c r="A39" s="11" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>生物</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>10-28 生物作业：第二章知识加油站 选择题</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>第12题</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>结构层次的判定（种子=器官）</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>把棉花种子当成植物体（因为种子能长成植株），误选水稻</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>正确 C 油菜花。种子是器官；水稻、苔藓是植物体，番茄果肉是组织</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>❌未掌握</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
       <c r="J39" s="2" t="n"/>
       <c r="K39" s="4" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="n"/>
-      <c r="B40" s="2" t="n"/>
-      <c r="C40" s="2" t="n"/>
-      <c r="D40" s="2" t="n"/>
-      <c r="E40" s="4" t="n"/>
-      <c r="F40" s="4" t="n"/>
-      <c r="G40" s="4" t="n"/>
-      <c r="H40" s="2" t="n"/>
-      <c r="I40" s="2" t="n"/>
+      <c r="A40" s="11" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>生物</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>10-28 生物作业：第二章知识加油站 选择题</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>第16题</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>器官与组织的区分（种子、鳃都是器官）</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>未识别D项错误（把种子、鳃当成组织），误选A</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>正确 D。种子=器官，鳃=器官；A项「都由受精卵发育而来」是对的</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>❌未掌握</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
       <c r="J40" s="2" t="n"/>
       <c r="K40" s="4" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="n"/>
-      <c r="B41" s="2" t="n"/>
-      <c r="C41" s="2" t="n"/>
-      <c r="D41" s="2" t="n"/>
-      <c r="E41" s="4" t="n"/>
-      <c r="F41" s="4" t="n"/>
-      <c r="G41" s="4" t="n"/>
-      <c r="H41" s="2" t="n"/>
-      <c r="I41" s="2" t="n"/>
+      <c r="A41" s="11" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>生物</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>10-28 生物作业：第二章知识加油站 选择题</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>第23题</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>植物食用器官的辨识（根/茎/叶/花/果/种子）</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>胡萝卜误判为茎（实为根）；未识别番茄=果实的正确项</t>
+        </is>
+      </c>
+      <c r="G41" s="4" t="inlineStr">
+        <is>
+          <t>正确 A 番茄—果实。胡萝卜=肉质直根；花椰菜=花；油菜=叶和茎</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>❌未掌握</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
       <c r="J41" s="2" t="n"/>
       <c r="K41" s="4" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="n"/>
-      <c r="B42" s="2" t="n"/>
-      <c r="C42" s="2" t="n"/>
-      <c r="D42" s="2" t="n"/>
-      <c r="E42" s="4" t="n"/>
-      <c r="F42" s="4" t="n"/>
-      <c r="G42" s="4" t="n"/>
-      <c r="H42" s="2" t="n"/>
-      <c r="I42" s="2" t="n"/>
+      <c r="A42" s="11" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>生物</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>10-28 生物作业：第二章知识加油站 非选择题</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>第32题(1) 染色体数目</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>细胞分裂后染色体数目不变（复制后平分）</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
+          <t>填「加倍」，只记住复制这一步，漏掉平分</t>
+        </is>
+      </c>
+      <c r="G42" s="4" t="inlineStr">
+        <is>
+          <t>正确「不变」。复制后平均分入两个新细胞，子细胞染色体数=原细胞（46条）</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>❌未掌握</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
       <c r="J42" s="2" t="n"/>
       <c r="K42" s="4" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="n"/>
-      <c r="B43" s="2" t="n"/>
-      <c r="C43" s="2" t="n"/>
-      <c r="D43" s="2" t="n"/>
-      <c r="E43" s="4" t="n"/>
-      <c r="F43" s="4" t="n"/>
-      <c r="G43" s="4" t="n"/>
-      <c r="H43" s="2" t="n"/>
-      <c r="I43" s="2" t="n"/>
+      <c r="A43" s="11" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>生物</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>10-28 生物作业：第二章知识加油站 非选择题</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>第32题(3) 胃出血对应组织</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>血液属于结缔组织</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>把胃出血归到上皮组织（表面保护），未联系到血液=结缔组织</t>
+        </is>
+      </c>
+      <c r="G43" s="4" t="inlineStr">
+        <is>
+          <t>正确「结缔组织」。蠕动=肌肉、疼痛=神经、出血=结缔（血液）</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>❌未掌握</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
       <c r="J43" s="2" t="n"/>
       <c r="K43" s="4" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="n"/>
-      <c r="B44" s="2" t="n"/>
-      <c r="C44" s="2" t="n"/>
-      <c r="D44" s="2" t="n"/>
-      <c r="E44" s="4" t="n"/>
-      <c r="F44" s="4" t="n"/>
-      <c r="G44" s="4" t="n"/>
-      <c r="H44" s="2" t="n"/>
-      <c r="I44" s="2" t="n"/>
+      <c r="A44" s="11" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>生物</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>10-28 生物作业：第二章知识加油站 非选择题</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>第32题(4) 人体特有层次</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>人体特有结构层次=系统（植物无系统）</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
+          <t>选C（个体），未提取图中B=消化系统</t>
+        </is>
+      </c>
+      <c r="G44" s="4" t="inlineStr">
+        <is>
+          <t>正确 B（系统）。图A=胃(器官)、B=消化系统(系统)、C=人(个体)</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>❌未掌握</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
       <c r="J44" s="2" t="n"/>
       <c r="K44" s="4" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="n"/>
-      <c r="B45" s="2" t="n"/>
-      <c r="C45" s="2" t="n"/>
-      <c r="D45" s="2" t="n"/>
-      <c r="E45" s="4" t="n"/>
-      <c r="F45" s="4" t="n"/>
-      <c r="G45" s="4" t="n"/>
-      <c r="H45" s="2" t="n"/>
-      <c r="I45" s="2" t="n"/>
+      <c r="A45" s="11" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>生物</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>10-28 生物作业：第二章知识加油站 非选择题</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>第34题(2) 草履虫体内绿色结构</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>草履虫无异养动物，无叶绿体；吞入的叶绿体在食物泡中</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>把草履虫当成植物，写了「叶绿体」</t>
+        </is>
+      </c>
+      <c r="G45" s="4" t="inlineStr">
+        <is>
+          <t>正确「食物泡」。草履虫是单细胞动物，不能光合作用；眼虫才有叶绿体</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>❌未掌握</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
       <c r="J45" s="2" t="n"/>
       <c r="K45" s="4" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="n"/>
-      <c r="B46" s="2" t="n"/>
-      <c r="C46" s="2" t="n"/>
-      <c r="D46" s="2" t="n"/>
-      <c r="E46" s="4" t="n"/>
-      <c r="F46" s="4" t="n"/>
-      <c r="G46" s="4" t="n"/>
-      <c r="H46" s="2" t="n"/>
-      <c r="I46" s="2" t="n"/>
+      <c r="A46" s="11" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>英语</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>蓝天宝典 U1 词性转换默写（P11）</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>第3组 improve</t>
+        </is>
+      </c>
+      <c r="E46" s="4" t="inlineStr">
+        <is>
+          <t>improve(v.) → improvement(n.) 进步、改善</t>
+        </is>
+      </c>
+      <c r="F46" s="4" t="inlineStr">
+        <is>
+          <t>把原词 improve 又抄一遍，没注意题目要的是名词形式</t>
+        </is>
+      </c>
+      <c r="G46" s="4" t="inlineStr">
+        <is>
+          <t>动词 + -ment 变名词。同类：develop→development、move→movement、agree→agreement、achieve→achievement</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>❌未掌握</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
       <c r="J46" s="2" t="n"/>
       <c r="K46" s="4" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="n"/>
-      <c r="B47" s="2" t="n"/>
-      <c r="C47" s="2" t="n"/>
-      <c r="D47" s="2" t="n"/>
-      <c r="E47" s="4" t="n"/>
-      <c r="F47" s="4" t="n"/>
-      <c r="G47" s="4" t="n"/>
-      <c r="H47" s="2" t="n"/>
-      <c r="I47" s="2" t="n"/>
+      <c r="A47" s="11" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>数学</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 福田区石厦学校七上期中数学模拟卷（67/100，班均69.98）</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>选择题6</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>整体代入求值（含字母表示负数）</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>转念/最后一步：只算了 a²−2b=−10 的一半，没走完 (乘−2再+15)；且误判 −m 一定为负数</t>
+        </is>
+      </c>
+      <c r="G47" s="4" t="inlineStr">
+        <is>
+          <t>B：由 a²−2b=5 乘 −2 得 −2a²+4b=−10，+15=5；A 错在 m 可为负数</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>❌未掌握</t>
+        </is>
+      </c>
+      <c r="I47" s="11" t="n">
+        <v>46326</v>
+      </c>
       <c r="J47" s="2" t="n"/>
-      <c r="K47" s="4" t="n"/>
+      <c r="K47" s="4" t="inlineStr">
+        <is>
+          <t>D+2(10/31 周六专项)、D+5(11/03)、D+8(11/06 期中)</t>
+        </is>
+      </c>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="n"/>
-      <c r="B48" s="2" t="n"/>
-      <c r="C48" s="2" t="n"/>
-      <c r="D48" s="2" t="n"/>
-      <c r="E48" s="4" t="n"/>
-      <c r="F48" s="4" t="n"/>
-      <c r="G48" s="4" t="n"/>
-      <c r="H48" s="2" t="n"/>
-      <c r="I48" s="2" t="n"/>
+      <c r="A48" s="11" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>数学</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 福田区石厦学校七上期中数学模拟卷（67/100，班均69.98）</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>选择题7</t>
+        </is>
+      </c>
+      <c r="E48" s="4" t="inlineStr">
+        <is>
+          <t>面动成体（矩形绕边旋转成圆柱）</t>
+        </is>
+      </c>
+      <c r="F48" s="4" t="inlineStr">
+        <is>
+          <t>不会（空间想象未建立）：没把旋转想象成圆柱，直接放弃空白</t>
+        </is>
+      </c>
+      <c r="G48" s="4" t="inlineStr">
+        <is>
+          <t>D：绕右边转，半径=宽=2r，V=π(2r)²h=4πr²h</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>❌未掌握</t>
+        </is>
+      </c>
+      <c r="I48" s="11" t="n">
+        <v>46326</v>
+      </c>
       <c r="J48" s="2" t="n"/>
-      <c r="K48" s="4" t="n"/>
+      <c r="K48" s="4" t="inlineStr">
+        <is>
+          <t>D+2(10/31 周六专项)、D+5(11/03)、D+8(11/06 期中)</t>
+        </is>
+      </c>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="n"/>
-      <c r="B49" s="2" t="n"/>
-      <c r="C49" s="2" t="n"/>
-      <c r="D49" s="2" t="n"/>
-      <c r="E49" s="4" t="n"/>
-      <c r="F49" s="4" t="n"/>
-      <c r="G49" s="4" t="n"/>
-      <c r="H49" s="2" t="n"/>
-      <c r="I49" s="2" t="n"/>
+      <c r="A49" s="11" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>数学</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 福田区石厦学校七上期中数学模拟卷（67/100，班均69.98）</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>填空题11</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="inlineStr">
+        <is>
+          <t>整式与 x、y 无关求参数</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>最后一步：整理出 (2m+8)x²+(3−n)y−5 后，最后一步 (−1)^2025 算错</t>
+        </is>
+      </c>
+      <c r="G49" s="4" t="inlineStr">
+        <is>
+          <t>m=−4、n=3 ⇒ m+n=−1 ⇒ (−1)^2025=−1</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>❌未掌握</t>
+        </is>
+      </c>
+      <c r="I49" s="11" t="n">
+        <v>46326</v>
+      </c>
       <c r="J49" s="2" t="n"/>
-      <c r="K49" s="4" t="n"/>
+      <c r="K49" s="4" t="inlineStr">
+        <is>
+          <t>D+2(10/31 周六专项)、D+5(11/03)、D+8(11/06 期中)</t>
+        </is>
+      </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="n"/>
-      <c r="B50" s="2" t="n"/>
-      <c r="C50" s="2" t="n"/>
-      <c r="D50" s="2" t="n"/>
-      <c r="E50" s="4" t="n"/>
-      <c r="F50" s="4" t="n"/>
-      <c r="G50" s="4" t="n"/>
-      <c r="H50" s="2" t="n"/>
-      <c r="I50" s="2" t="n"/>
+      <c r="A50" s="11" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>数学</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 福田区石厦学校七上期中数学模拟卷（67/100，班均69.98）</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>填空题13</t>
+        </is>
+      </c>
+      <c r="E50" s="4" t="inlineStr">
+        <is>
+          <t>程序框图周期性规律</t>
+        </is>
+      </c>
+      <c r="F50" s="4" t="inlineStr">
+        <is>
+          <t>规律题流程缺失：未列出足够输出项找周期，末项算错</t>
+        </is>
+      </c>
+      <c r="G50" s="4" t="inlineStr">
+        <is>
+          <t>输出 1,−4,−2,−1,−6,−3,−8,−4…周期6 ⇒ 第2026次=−1</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>❌未掌握</t>
+        </is>
+      </c>
+      <c r="I50" s="11" t="n">
+        <v>46326</v>
+      </c>
       <c r="J50" s="2" t="n"/>
-      <c r="K50" s="4" t="n"/>
+      <c r="K50" s="4" t="inlineStr">
+        <is>
+          <t>D+2(10/31 周六专项)、D+5(11/03)、D+8(11/06 期中)</t>
+        </is>
+      </c>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="n"/>
-      <c r="B51" s="2" t="n"/>
-      <c r="C51" s="2" t="n"/>
-      <c r="D51" s="2" t="n"/>
-      <c r="E51" s="4" t="n"/>
-      <c r="F51" s="4" t="n"/>
-      <c r="G51" s="4" t="n"/>
-      <c r="H51" s="2" t="n"/>
-      <c r="I51" s="2" t="n"/>
+      <c r="A51" s="11" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>数学</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 福田区石厦学校七上期中数学模拟卷（67/100，班均69.98）</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>15（6分）</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="inlineStr">
+        <is>
+          <t>先化简再求值（格式）</t>
+        </is>
+      </c>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
+          <t>书写规范：过程和答案全对（2ab²=18），但缺「解：」「当 a=1，b=−3 时，」，被判格式错</t>
+        </is>
+      </c>
+      <c r="G51" s="4" t="inlineStr">
+        <is>
+          <t>标准格式：解：原式=…=2ab²；当 a=1，b=−3 时，原式=2×1×(−3)²=18</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>❌未掌握</t>
+        </is>
+      </c>
+      <c r="I51" s="11" t="n">
+        <v>46326</v>
+      </c>
       <c r="J51" s="2" t="n"/>
-      <c r="K51" s="4" t="n"/>
+      <c r="K51" s="4" t="inlineStr">
+        <is>
+          <t>D+2(10/31 周六专项)、D+5(11/03)、D+8(11/06 期中)</t>
+        </is>
+      </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="n"/>
-      <c r="B52" s="2" t="n"/>
-      <c r="C52" s="2" t="n"/>
-      <c r="D52" s="2" t="n"/>
-      <c r="E52" s="4" t="n"/>
-      <c r="F52" s="4" t="n"/>
-      <c r="G52" s="4" t="n"/>
-      <c r="H52" s="2" t="n"/>
-      <c r="I52" s="2" t="n"/>
+      <c r="A52" s="11" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>数学</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 福田区石厦学校七上期中数学模拟卷（67/100，班均69.98）</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>16(2)（2分）</t>
+        </is>
+      </c>
+      <c r="E52" s="4" t="inlineStr">
+        <is>
+          <t>三视图「最多添加小正方体」</t>
+        </is>
+      </c>
+      <c r="F52" s="4" t="inlineStr">
+        <is>
+          <t>方法未掌握：只凭数感填2，未列上限矩阵 min(该列正视高度, 该行左视高度)</t>
+        </is>
+      </c>
+      <c r="G52" s="4" t="inlineStr">
+        <is>
+          <t>标准答案 4：上限表（正视3,1,2 × 左视3,2,1）逐格取min ⇒ 3,1,2 / 2,1,2 / 1,1,1 合计 14；现有 10 个，最多再添加 4 个</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>❌未掌握</t>
+        </is>
+      </c>
+      <c r="I52" s="11" t="n">
+        <v>46326</v>
+      </c>
       <c r="J52" s="2" t="n"/>
-      <c r="K52" s="4" t="n"/>
+      <c r="K52" s="4" t="inlineStr">
+        <is>
+          <t>D+2(10/31 周六专项)、D+5(11/03)、D+8(11/06 期中)</t>
+        </is>
+      </c>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="n"/>
-      <c r="B53" s="2" t="n"/>
-      <c r="C53" s="2" t="n"/>
-      <c r="D53" s="2" t="n"/>
-      <c r="E53" s="4" t="n"/>
-      <c r="F53" s="4" t="n"/>
-      <c r="G53" s="4" t="n"/>
-      <c r="H53" s="2" t="n"/>
-      <c r="I53" s="2" t="n"/>
+      <c r="A53" s="11" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>数学</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 福田区石厦学校七上期中数学模拟卷（67/100，班均69.98）</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>17(3)（2分）</t>
+        </is>
+      </c>
+      <c r="E53" s="4" t="inlineStr">
+        <is>
+          <t>有理数应用题·油耗计算</t>
+        </is>
+      </c>
+      <c r="F53" s="4" t="inlineStr">
+        <is>
+          <t>最后一步/抄错数：357÷100=3.57 后把 3.57 抄成 3.56，算出 21.36</t>
+        </is>
+      </c>
+      <c r="G53" s="4" t="inlineStr">
+        <is>
+          <t>357÷100×6=21.42 升</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>❌未掌握</t>
+        </is>
+      </c>
+      <c r="I53" s="11" t="n">
+        <v>46326</v>
+      </c>
       <c r="J53" s="2" t="n"/>
-      <c r="K53" s="4" t="n"/>
+      <c r="K53" s="4" t="inlineStr">
+        <is>
+          <t>D+2(10/31 周六专项)、D+5(11/03)、D+8(11/06 期中)</t>
+        </is>
+      </c>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="n"/>
-      <c r="B54" s="2" t="n"/>
-      <c r="C54" s="2" t="n"/>
-      <c r="D54" s="2" t="n"/>
-      <c r="E54" s="4" t="n"/>
-      <c r="F54" s="4" t="n"/>
-      <c r="G54" s="4" t="n"/>
-      <c r="H54" s="2" t="n"/>
-      <c r="I54" s="2" t="n"/>
+      <c r="A54" s="11" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>数学</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 福田区石厦学校七上期中数学模拟卷（67/100，班均69.98）</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>18(2)①（1分）</t>
+        </is>
+      </c>
+      <c r="E54" s="4" t="inlineStr">
+        <is>
+          <t>幂的差（1−2⁶）</t>
+        </is>
+      </c>
+      <c r="F54" s="4" t="inlineStr">
+        <is>
+          <t>最后一步：算出 2⁶=64 后忘了 1−64=−63，写 −64</t>
+        </is>
+      </c>
+      <c r="G54" s="4" t="inlineStr">
+        <is>
+          <t>1−2⁶=−63</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>❌未掌握</t>
+        </is>
+      </c>
+      <c r="I54" s="11" t="n">
+        <v>46326</v>
+      </c>
       <c r="J54" s="2" t="n"/>
-      <c r="K54" s="4" t="n"/>
+      <c r="K54" s="4" t="inlineStr">
+        <is>
+          <t>D+2(10/31 周六专项)、D+5(11/03)、D+8(11/06 期中)</t>
+        </is>
+      </c>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="n"/>
-      <c r="B55" s="2" t="n"/>
-      <c r="C55" s="2" t="n"/>
-      <c r="D55" s="2" t="n"/>
-      <c r="E55" s="4" t="n"/>
-      <c r="F55" s="4" t="n"/>
-      <c r="G55" s="4" t="n"/>
-      <c r="H55" s="2" t="n"/>
-      <c r="I55" s="2" t="n"/>
+      <c r="A55" s="11" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>数学</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 福田区石厦学校七上期中数学模拟卷（67/100，班均69.98）</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>18(2)②（1分）</t>
+        </is>
+      </c>
+      <c r="E55" s="4" t="inlineStr">
+        <is>
+          <t>多项式乘法反向（x−1 型）</t>
+        </is>
+      </c>
+      <c r="F55" s="4" t="inlineStr">
+        <is>
+          <t>符号方向：答案写成 1−x²⁰²³，符号方向反</t>
+        </is>
+      </c>
+      <c r="G55" s="4" t="inlineStr">
+        <is>
+          <t>(x−1)(x²⁰²²+…+1)=x²⁰²³−1</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>❌未掌握</t>
+        </is>
+      </c>
+      <c r="I55" s="11" t="n">
+        <v>46326</v>
+      </c>
       <c r="J55" s="2" t="n"/>
-      <c r="K55" s="4" t="n"/>
+      <c r="K55" s="4" t="inlineStr">
+        <is>
+          <t>D+2(10/31 周六专项)、D+5(11/03)、D+8(11/06 期中)</t>
+        </is>
+      </c>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="n"/>
-      <c r="B56" s="2" t="n"/>
-      <c r="C56" s="2" t="n"/>
-      <c r="D56" s="2" t="n"/>
-      <c r="E56" s="4" t="n"/>
-      <c r="F56" s="4" t="n"/>
-      <c r="G56" s="4" t="n"/>
-      <c r="H56" s="2" t="n"/>
-      <c r="I56" s="2" t="n"/>
+      <c r="A56" s="11" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>数学</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 福田区石厦学校七上期中数学模拟卷（67/100，班均69.98）</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>18(3)（1分）</t>
+        </is>
+      </c>
+      <c r="E56" s="4" t="inlineStr">
+        <is>
+          <t>等比数列求和（迁移应用）</t>
+        </is>
+      </c>
+      <c r="F56" s="4" t="inlineStr">
+        <is>
+          <t>不提笔到底：只抄了 2¹⁰⁰+2⁹⁹+… 的式子，未求值</t>
+        </is>
+      </c>
+      <c r="G56" s="4" t="inlineStr">
+        <is>
+          <t>2¹⁰⁰+…+1=(2−1)(2¹⁰⁰+…+1)=2¹⁰¹−1</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>❌未掌握</t>
+        </is>
+      </c>
+      <c r="I56" s="11" t="n">
+        <v>46326</v>
+      </c>
       <c r="J56" s="2" t="n"/>
-      <c r="K56" s="4" t="n"/>
+      <c r="K56" s="4" t="inlineStr">
+        <is>
+          <t>D+2(10/31 周六专项)、D+5(11/03)、D+8(11/06 期中)</t>
+        </is>
+      </c>
     </row>
     <row r="57">
-      <c r="A57" s="2" t="n"/>
-      <c r="B57" s="2" t="n"/>
-      <c r="C57" s="2" t="n"/>
-      <c r="D57" s="2" t="n"/>
-      <c r="E57" s="4" t="n"/>
-      <c r="F57" s="4" t="n"/>
-      <c r="G57" s="4" t="n"/>
-      <c r="H57" s="2" t="n"/>
-      <c r="I57" s="2" t="n"/>
+      <c r="A57" s="11" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>数学</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 福田区石厦学校七上期中数学模拟卷（67/100，班均69.98）</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>19 问题三（1分）</t>
+        </is>
+      </c>
+      <c r="E57" s="4" t="inlineStr">
+        <is>
+          <t>分段计费/分类比较</t>
+        </is>
+      </c>
+      <c r="F57" s="4" t="inlineStr">
+        <is>
+          <t>最后一步/加总错：甲的总价合计多加 100（17760 应 17660），结论未受影响</t>
+        </is>
+      </c>
+      <c r="G57" s="4" t="inlineStr">
+        <is>
+          <t>4000+10780+2880=17660；乙 17000 &lt; 17660 ⇒ 乙更划算</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>❌未掌握</t>
+        </is>
+      </c>
+      <c r="I57" s="11" t="n">
+        <v>46326</v>
+      </c>
       <c r="J57" s="2" t="n"/>
-      <c r="K57" s="4" t="n"/>
+      <c r="K57" s="4" t="inlineStr">
+        <is>
+          <t>D+2(10/31 周六专项)、D+5(11/03)、D+8(11/06 期中)</t>
+        </is>
+      </c>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="n"/>
-      <c r="B58" s="2" t="n"/>
-      <c r="C58" s="2" t="n"/>
-      <c r="D58" s="2" t="n"/>
-      <c r="E58" s="4" t="n"/>
-      <c r="F58" s="4" t="n"/>
-      <c r="G58" s="4" t="n"/>
-      <c r="H58" s="2" t="n"/>
-      <c r="I58" s="2" t="n"/>
+      <c r="A58" s="11" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>数学</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 福田区石厦学校七上期中数学模拟卷（67/100，班均69.98）</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>20(3)（3分）</t>
+        </is>
+      </c>
+      <c r="E58" s="4" t="inlineStr">
+        <is>
+          <t>数轴动点：用含 t 的式子表示点</t>
+        </is>
+      </c>
+      <c r="F58" s="4" t="inlineStr">
+        <is>
+          <t>不信任自己的正确写法：P=−4+x 写对后自己划掉；Q 写 −2x 漏起点 16</t>
+        </is>
+      </c>
+      <c r="G58" s="4" t="inlineStr">
+        <is>
+          <t>P=x−4；Q=16−2x</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>❌未掌握</t>
+        </is>
+      </c>
+      <c r="I58" s="11" t="n">
+        <v>46326</v>
+      </c>
       <c r="J58" s="2" t="n"/>
-      <c r="K58" s="4" t="n"/>
+      <c r="K58" s="4" t="inlineStr">
+        <is>
+          <t>D+2(10/31 周六专项)、D+5(11/03)、D+8(11/06 期中)</t>
+        </is>
+      </c>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="n"/>
-      <c r="B59" s="2" t="n"/>
-      <c r="C59" s="2" t="n"/>
-      <c r="D59" s="2" t="n"/>
-      <c r="E59" s="4" t="n"/>
-      <c r="F59" s="4" t="n"/>
-      <c r="G59" s="4" t="n"/>
-      <c r="H59" s="2" t="n"/>
-      <c r="I59" s="2" t="n"/>
+      <c r="A59" s="11" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>数学</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 福田区石厦学校七上期中数学模拟卷（67/100，班均69.98）</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>20(4)（5分）</t>
+        </is>
+      </c>
+      <c r="E59" s="4" t="inlineStr">
+        <is>
+          <t>数轴动点·先后出发与绝对值</t>
+        </is>
+      </c>
+      <c r="F59" s="4" t="inlineStr">
+        <is>
+          <t>动点五步法未建立：两个方程都丢起点、无绝对值、未区分 Q 先走 2 秒</t>
+        </is>
+      </c>
+      <c r="G59" s="4" t="inlineStr">
+        <is>
+          <t>Q=16−2t，P=t−6，|22−3t|=5 ⇒ t=17/3 或 9</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>❌未掌握</t>
+        </is>
+      </c>
+      <c r="I59" s="11" t="n">
+        <v>46326</v>
+      </c>
       <c r="J59" s="2" t="n"/>
-      <c r="K59" s="4" t="n"/>
+      <c r="K59" s="4" t="inlineStr">
+        <is>
+          <t>D+2(10/31 周六专项)、D+5(11/03)、D+8(11/06 期中)</t>
+        </is>
+      </c>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="n"/>
-      <c r="B60" s="2" t="n"/>
-      <c r="C60" s="2" t="n"/>
-      <c r="D60" s="2" t="n"/>
-      <c r="E60" s="4" t="n"/>
-      <c r="F60" s="4" t="n"/>
-      <c r="G60" s="4" t="n"/>
-      <c r="H60" s="2" t="n"/>
-      <c r="I60" s="2" t="n"/>
+      <c r="A60" s="11" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>历史</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 第9课 秦统一中国 课时练习（家长转图）</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>第9课 选择01（AI诗选标题）</t>
+        </is>
+      </c>
+      <c r="E60" s="4" t="inlineStr">
+        <is>
+          <t>秦统一中国·诗句与史实对应</t>
+        </is>
+      </c>
+      <c r="F60" s="4" t="inlineStr">
+        <is>
+          <t>未抓关键词「六国尽扫平、书同文字」→未想到秦统一</t>
+        </is>
+      </c>
+      <c r="G60" s="4" t="inlineStr">
+        <is>
+          <t>C．《咏秦》</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>❌未掌握</t>
+        </is>
+      </c>
+      <c r="I60" s="11" t="n">
+        <v>46326</v>
+      </c>
       <c r="J60" s="2" t="n"/>
-      <c r="K60" s="4" t="n"/>
+      <c r="K60" s="4" t="inlineStr">
+        <is>
+          <t>D+2(10/31)、D+5(11/03)、D+8(11/06 期中)</t>
+        </is>
+      </c>
     </row>
     <row r="61">
-      <c r="A61" s="2" t="n"/>
-      <c r="B61" s="2" t="n"/>
-      <c r="C61" s="2" t="n"/>
-      <c r="D61" s="2" t="n"/>
-      <c r="E61" s="4" t="n"/>
-      <c r="F61" s="4" t="n"/>
-      <c r="G61" s="4" t="n"/>
-      <c r="H61" s="2" t="n"/>
-      <c r="I61" s="2" t="n"/>
+      <c r="A61" s="11" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>历史</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 第9课 秦统一中国 课时练习（家长转图）</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>第9课 选择02（王夫之《读通鉴论》）</t>
+        </is>
+      </c>
+      <c r="E61" s="4" t="inlineStr">
+        <is>
+          <t>郡县制·顺应历史发展趋势</t>
+        </is>
+      </c>
+      <c r="F61" s="4" t="inlineStr">
+        <is>
+          <t>未抓「势之所趋、二千年弗能改」→把「作用」当成「趋势」</t>
+        </is>
+      </c>
+      <c r="G61" s="4" t="inlineStr">
+        <is>
+          <t>C．顺应历史趋势</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>❌未掌握</t>
+        </is>
+      </c>
+      <c r="I61" s="11" t="n">
+        <v>46326</v>
+      </c>
       <c r="J61" s="2" t="n"/>
-      <c r="K61" s="4" t="n"/>
+      <c r="K61" s="4" t="inlineStr">
+        <is>
+          <t>D+2(10/31)、D+5(11/03)、D+8(11/06 期中)</t>
+        </is>
+      </c>
     </row>
     <row r="62">
-      <c r="A62" s="2" t="n"/>
-      <c r="B62" s="2" t="n"/>
-      <c r="C62" s="2" t="n"/>
-      <c r="D62" s="2" t="n"/>
-      <c r="E62" s="4" t="n"/>
-      <c r="F62" s="4" t="n"/>
-      <c r="G62" s="4" t="n"/>
-      <c r="H62" s="2" t="n"/>
-      <c r="I62" s="2" t="n"/>
+      <c r="A62" s="11" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>历史</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 第9课 秦统一中国 课时练习（家长转图）</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>第9课 选择03（秦直道700km/两年半）</t>
+        </is>
+      </c>
+      <c r="E62" s="4" t="inlineStr">
+        <is>
+          <t>秦巩固统一措施·国家体制的作用</t>
+        </is>
+      </c>
+      <c r="F62" s="4" t="inlineStr">
+        <is>
+          <t>只看「修路」误选技术；忽略「规模大速度快」=中央集权组织能力</t>
+        </is>
+      </c>
+      <c r="G62" s="4" t="inlineStr">
+        <is>
+          <t>C．国家体制的作用</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>❌未掌握</t>
+        </is>
+      </c>
+      <c r="I62" s="11" t="n">
+        <v>46326</v>
+      </c>
       <c r="J62" s="2" t="n"/>
-      <c r="K62" s="4" t="n"/>
+      <c r="K62" s="4" t="inlineStr">
+        <is>
+          <t>D+2(10/31)、D+5(11/03)、D+8(11/06 期中)</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n"/>

</xml_diff>